<commit_message>
Give the kitchen sink sample Excel 365 checkboxes, written by XlsxWriter: a Reviewed tick per region and one worked out from them
</commit_message>
<xml_diff>
--- a/examples/demo/public/samples/kitchen-sink.xlsx
+++ b/examples/demo/public/samples/kitchen-sink.xlsx
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="64">
   <si>
     <t>Tax rate</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>Share</t>
+  </si>
+  <si>
+    <t>Reviewed</t>
   </si>
   <si>
     <t>Tax due</t>
@@ -409,7 +412,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -418,6 +421,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1039,6 +1049,23 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SalesData" displayName="SalesData" ref="A1:F201" totalsRowShown="0">
   <autoFilter ref="A1:F201"/>
@@ -1339,7 +1366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -1347,7 +1374,7 @@
     <col min="7" max="7" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -1358,7 +1385,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1371,10 +1398,10 @@
       </c>
       <c r="E2" s="2">
         <f>TODAY()</f>
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1396,8 +1423,11 @@
       <c r="G4" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1425,8 +1455,11 @@
         <f>F5/$F$9</f>
         <v>0.23023234093344794</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1454,8 +1487,11 @@
         <f>F6/$F$9</f>
         <v>0.27007239184360954</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1483,8 +1519,11 @@
         <f>F7/$F$9</f>
         <v>0.26792580667119414</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1512,37 +1551,44 @@
         <f>F8/$F$9</f>
         <v>0.23176946055174838</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="6" t="s">
+      <c r="H8" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="8">
         <f>SUM(B5:B8)</f>
         <v>38888.0</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="8">
         <f>SUM(C5:C8)</f>
         <v>34882.0</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="8">
         <f>SUM(D5:D8)</f>
         <v>29862.5</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="8">
         <f>SUM(E5:E8)</f>
         <v>54292.75</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="8">
         <f>SUM(F5:F8)</f>
         <v>157925.25</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="9">
         <f>SUM(G5:G8)</f>
         <v>1.0</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H9" s="6" t="b">
+        <f>AND(H5:H8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1551,45 +1597,45 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="4">
         <f>F9*TaxRate</f>
         <v>31585.050000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" t="str">
         <f>INDEX(A5:A8,MATCH(MAX(F5:F8),F5:F8,0))</f>
         <v>South</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,A5:A8)</f>
         <v>North, South, East, West</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" t="str">
         <f>_xlfn.CONCAT(A5:A8)</f>
         <v>NorthSouthEastWest</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="4">
         <f>_xlfn.LET(revenue,F9,cost,F9*0.6,revenue-cost)</f>
@@ -1598,7 +1644,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="4">
         <f>B16*(1-TaxRate)</f>
@@ -1606,20 +1652,20 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="9" t="s">
-        <v>29</v>
+      <c r="A19" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="10">
+      <c r="A22" s="11">
         <v>46023</v>
       </c>
       <c r="B22" s="4">
@@ -1628,7 +1674,7 @@
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="10">
+      <c r="A23" s="11">
         <v>46054</v>
       </c>
       <c r="B23" s="4">
@@ -1637,7 +1683,7 @@
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="10">
+      <c r="A24" s="11">
         <v>46082</v>
       </c>
       <c r="B24" s="4">
@@ -1646,7 +1692,7 @@
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="10">
+      <c r="A25" s="11">
         <v>46113</v>
       </c>
       <c r="B25" s="4">
@@ -1655,7 +1701,7 @@
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="10">
+      <c r="A26" s="11">
         <v>46143</v>
       </c>
       <c r="B26" s="4">
@@ -1664,7 +1710,7 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="10">
+      <c r="A27" s="11">
         <v>46174</v>
       </c>
       <c r="B27" s="4">
@@ -1673,7 +1719,7 @@
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="10">
+      <c r="A28" s="11">
         <v>46204</v>
       </c>
       <c r="B28" s="4">
@@ -1682,7 +1728,7 @@
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="10">
+      <c r="A29" s="11">
         <v>46235</v>
       </c>
       <c r="B29" s="4">
@@ -1691,7 +1737,7 @@
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="10">
+      <c r="A30" s="11">
         <v>46266</v>
       </c>
       <c r="B30" s="4">
@@ -1700,7 +1746,7 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="10">
+      <c r="A31" s="11">
         <v>46296</v>
       </c>
       <c r="B31" s="4">
@@ -1709,7 +1755,7 @@
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="10">
+      <c r="A32" s="11">
         <v>46327</v>
       </c>
       <c r="B32" s="4">
@@ -1718,7 +1764,7 @@
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="10">
+      <c r="A33" s="11">
         <v>46357</v>
       </c>
       <c r="B33" s="4">
@@ -6003,8 +6049,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="6" t="s">
-        <v>31</v>
+      <c r="A1" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -6012,13 +6058,13 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>3</v>
@@ -6098,7 +6144,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" s="4">
         <f>SUM(SalesData[Revenue])</f>
@@ -6107,7 +6153,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" cm="1" t="str">
         <f t="array" ref="B9:B12">_xlfn._xlws.SORT(_xlfn.UNIQUE(Data!B2:B201))</f>
@@ -6131,7 +6177,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" s="4">
         <f t="array" ref="B14">SUM(Data!D2:D201*Data!E2:E201)</f>
@@ -6140,7 +6186,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="4">
         <f t="array" ref="B15:D15">TRANSPOSE(G4:G6*2)</f>
@@ -6155,15 +6201,15 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" t="str">
         <f>_xlfn.IFS(B4&gt;20,"High",B4&gt;10,"Mid",TRUE,"Low")</f>
@@ -6172,7 +6218,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="2">
         <f>EDATE(DATE(2026,1,31),1)</f>
@@ -6181,7 +6227,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B20" t="str">
         <f>UPPER(LEFT(A4,3))&amp;"-"&amp;TEXT(G4,"0.00")</f>
@@ -6190,9 +6236,9 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="11" t="str">
+        <v>45</v>
+      </c>
+      <c r="B21" s="12" t="str">
         <f>IF(SUM(D4:D6)&lt;0,"Negative","OK")</f>
         <v>OK</v>
       </c>
@@ -6211,76 +6257,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="6" t="s">
-        <v>45</v>
+      <c r="A1" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="A2" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
     </row>
     <row r="6" spans="1:6" hidden="1">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -6341,15 +6387,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -6357,7 +6403,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -6365,7 +6411,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -6373,7 +6419,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>

</xml_diff>